<commit_message>
volcando de la tabla al excel
</commit_message>
<xml_diff>
--- a/codigo/resultados/resultados_RS_cv_vs_test.xlsx
+++ b/codigo/resultados/resultados_RS_cv_vs_test.xlsx
@@ -1,20 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos_D\TESIS\armado tesina\codigo\resultados\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7044C9C6-314D-4D49-8E11-E6078D6FB135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$155</definedName>
+  </definedNames>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="190">
   <si>
     <t>Tecnica</t>
   </si>
@@ -527,13 +537,70 @@
   </si>
   <si>
     <t>-------</t>
+  </si>
+  <si>
+    <t>percentil_radio_densidad</t>
+  </si>
+  <si>
+    <t>percentil_riesgo</t>
+  </si>
+  <si>
+    <t>criterio_pureza</t>
+  </si>
+  <si>
+    <t>umbral_densidad</t>
+  </si>
+  <si>
+    <t>percentil_entropia</t>
+  </si>
+  <si>
+    <t>umbral_pureza_proporcion</t>
+  </si>
+  <si>
+    <t>percentil_isolation</t>
+  </si>
+  <si>
+    <t>entropia</t>
+  </si>
+  <si>
+    <t>0.80</t>
+  </si>
+  <si>
+    <t>proporcion</t>
+  </si>
+  <si>
+    <t>0.40</t>
+  </si>
+  <si>
+    <t>0.50</t>
+  </si>
+  <si>
+    <t>0.60</t>
+  </si>
+  <si>
+    <t>0.55</t>
+  </si>
+  <si>
+    <t>0.65</t>
+  </si>
+  <si>
+    <t>0.70</t>
+  </si>
+  <si>
+    <t>0.75</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -585,10 +652,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -596,13 +666,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -640,7 +718,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -674,6 +752,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -708,9 +787,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -883,11 +963,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L155"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -925,7 +1010,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -951,19 +1036,19 @@
         <v>170</v>
       </c>
       <c r="I2">
-        <v>0.7012824798334791</v>
+        <v>0.70128247983347913</v>
       </c>
       <c r="J2">
-        <v>0.7099611137654616</v>
+        <v>0.70996111376546156</v>
       </c>
       <c r="K2">
-        <v>0.8846252479912903</v>
+        <v>0.88462524799129028</v>
       </c>
       <c r="L2">
-        <v>0.8985389610389611</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>0.89853896103896114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -989,19 +1074,19 @@
         <v>170</v>
       </c>
       <c r="I3">
-        <v>0.729352220587751</v>
+        <v>0.72935222058775095</v>
       </c>
       <c r="J3">
-        <v>0.7401556380127808</v>
+        <v>0.74015563801278084</v>
       </c>
       <c r="K3">
-        <v>0.9087301587301587</v>
+        <v>0.90873015873015872</v>
       </c>
       <c r="L3">
         <v>0.9241071428571429</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1027,19 +1112,19 @@
         <v>170</v>
       </c>
       <c r="I4">
-        <v>0.7104159316931057</v>
+        <v>0.71041593169310568</v>
       </c>
       <c r="J4">
-        <v>0.7204568981742894</v>
+        <v>0.72045689817428937</v>
       </c>
       <c r="K4">
-        <v>0.8846252479912903</v>
+        <v>0.88462524799129028</v>
       </c>
       <c r="L4">
-        <v>0.8985389610389611</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>0.89853896103896114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1065,19 +1150,19 @@
         <v>170</v>
       </c>
       <c r="I5">
-        <v>0.7048266015846494</v>
+        <v>0.70482660158464938</v>
       </c>
       <c r="J5">
-        <v>0.7207972582972582</v>
+        <v>0.72079725829725816</v>
       </c>
       <c r="K5">
-        <v>0.8846252479912903</v>
+        <v>0.88462524799129028</v>
       </c>
       <c r="L5">
-        <v>0.8985389610389611</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>0.89853896103896114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1106,16 +1191,16 @@
         <v>0.7234730506746867</v>
       </c>
       <c r="J6">
-        <v>0.7380931766646053</v>
+        <v>0.73809317666460528</v>
       </c>
       <c r="K6">
-        <v>0.882051282051282</v>
+        <v>0.88205128205128203</v>
       </c>
       <c r="L6">
-        <v>0.9032738095238096</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <v>0.90327380952380965</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1141,19 +1226,19 @@
         <v>170</v>
       </c>
       <c r="I7">
-        <v>0.673907075211423</v>
+        <v>0.67390707521142301</v>
       </c>
       <c r="J7">
-        <v>0.6774203574203574</v>
+        <v>0.67742035742035744</v>
       </c>
       <c r="K7">
-        <v>0.8374039938556067</v>
+        <v>0.83740399385560671</v>
       </c>
       <c r="L7">
-        <v>0.8325396825396826</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <v>0.83253968253968258</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1179,19 +1264,19 @@
         <v>170</v>
       </c>
       <c r="I8">
-        <v>0.7820869146956103</v>
+        <v>0.78208691469561031</v>
       </c>
       <c r="J8">
-        <v>0.803939393939394</v>
+        <v>0.80393939393939395</v>
       </c>
       <c r="K8">
-        <v>0.8457678522194652</v>
+        <v>0.84576785221946515</v>
       </c>
       <c r="L8">
-        <v>0.876984126984127</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <v>0.87698412698412698</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1217,19 +1302,19 @@
         <v>170</v>
       </c>
       <c r="I9">
-        <v>0.7385824266983687</v>
+        <v>0.73858242669836871</v>
       </c>
       <c r="J9">
-        <v>0.7394444444444445</v>
+        <v>0.73944444444444446</v>
       </c>
       <c r="K9">
         <v>0.8490421455938697</v>
       </c>
       <c r="L9">
-        <v>0.8436507936507937</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+        <v>0.84365079365079365</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1255,19 +1340,19 @@
         <v>170</v>
       </c>
       <c r="I10">
-        <v>0.732484631677614</v>
+        <v>0.73248463167761402</v>
       </c>
       <c r="J10">
-        <v>0.7410101010101011</v>
+        <v>0.74101010101010112</v>
       </c>
       <c r="K10">
-        <v>0.8088122605363984</v>
+        <v>0.80881226053639843</v>
       </c>
       <c r="L10">
-        <v>0.8206349206349207</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+        <v>0.82063492063492072</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1293,19 +1378,19 @@
         <v>170</v>
       </c>
       <c r="I11">
-        <v>0.74371278192102</v>
+        <v>0.74371278192101997</v>
       </c>
       <c r="J11">
-        <v>0.7544444444444445</v>
+        <v>0.75444444444444447</v>
       </c>
       <c r="K11">
-        <v>0.8076861808044603</v>
+        <v>0.80768618080446031</v>
       </c>
       <c r="L11">
-        <v>0.8214285714285715</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
+        <v>0.82142857142857151</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1331,19 +1416,19 @@
         <v>170</v>
       </c>
       <c r="I12">
-        <v>0.3020909846706401</v>
+        <v>0.30209098467064011</v>
       </c>
       <c r="J12">
-        <v>0.3088831908831909</v>
+        <v>0.30888319088319088</v>
       </c>
       <c r="K12">
-        <v>0.172972972972973</v>
+        <v>0.17297297297297301</v>
       </c>
       <c r="L12">
-        <v>0.1939393939393939</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
+        <v>0.19393939393939391</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -1372,16 +1457,16 @@
         <v>0.3421138861138861</v>
       </c>
       <c r="J13">
-        <v>0.3489275362318841</v>
+        <v>0.34892753623188411</v>
       </c>
       <c r="K13">
-        <v>0.1984344422700587</v>
+        <v>0.19843444227005869</v>
       </c>
       <c r="L13">
-        <v>0.2164502164502164</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+        <v>0.21645021645021639</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1410,16 +1495,16 @@
         <v>0.271574399884911</v>
       </c>
       <c r="J14">
-        <v>0.2826905982905983</v>
+        <v>0.28269059829059828</v>
       </c>
       <c r="K14">
-        <v>0.1961389961389962</v>
+        <v>0.19613899613899621</v>
       </c>
       <c r="L14">
-        <v>0.2164502164502164</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
+        <v>0.21645021645021639</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1445,19 +1530,19 @@
         <v>170</v>
       </c>
       <c r="I15">
-        <v>0.2854623225329542</v>
+        <v>0.28546232253295423</v>
       </c>
       <c r="J15">
-        <v>0.2948461538461539</v>
+        <v>0.29484615384615392</v>
       </c>
       <c r="K15">
-        <v>0.1948630136986302</v>
+        <v>0.19486301369863021</v>
       </c>
       <c r="L15">
-        <v>0.2164502164502164</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
+        <v>0.21645021645021639</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -1483,19 +1568,19 @@
         <v>170</v>
       </c>
       <c r="I16">
-        <v>0.3557152730310625</v>
+        <v>0.35571527303106248</v>
       </c>
       <c r="J16">
-        <v>0.3558888888888889</v>
+        <v>0.35588888888888892</v>
       </c>
       <c r="K16">
-        <v>0.217936507936508</v>
+        <v>0.21793650793650801</v>
       </c>
       <c r="L16">
-        <v>0.2346320346320346</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
+        <v>0.23463203463203461</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -1521,19 +1606,19 @@
         <v>170</v>
       </c>
       <c r="I17">
-        <v>0.9625943362606083</v>
+        <v>0.96259433626060831</v>
       </c>
       <c r="J17">
-        <v>0.9426045711074634</v>
+        <v>0.94260457110746343</v>
       </c>
       <c r="K17">
-        <v>0.8548829504460598</v>
+        <v>0.85488295044605978</v>
       </c>
       <c r="L17">
-        <v>0.8570626453838133</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12">
+        <v>0.85706264538381327</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -1559,27 +1644,27 @@
         <v>170</v>
       </c>
       <c r="I18">
-        <v>0.9377083597057845</v>
+        <v>0.93770835970578448</v>
       </c>
       <c r="J18">
-        <v>0.9092140921409214</v>
+        <v>0.90921409214092141</v>
       </c>
       <c r="K18">
-        <v>0.8349676826899955</v>
+        <v>0.83496768268999555</v>
       </c>
       <c r="L18">
-        <v>0.9271254558505639</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12">
+        <v>0.92712545585056394</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
         <v>20</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D19">
         <v>57532</v>
@@ -1590,26 +1675,23 @@
       <c r="F19">
         <v>45932</v>
       </c>
-      <c r="G19" t="s">
-        <v>170</v>
-      </c>
-      <c r="H19" t="s">
-        <v>170</v>
+      <c r="H19">
+        <v>206831</v>
       </c>
       <c r="I19">
-        <v>0.9339254137501722</v>
+        <v>0.99996834278416125</v>
       </c>
       <c r="J19">
-        <v>0.9026375885608062</v>
+        <v>0.99996834541483337</v>
       </c>
       <c r="K19">
-        <v>0.8307270961145612</v>
+        <v>1</v>
       </c>
       <c r="L19">
-        <v>0.8564822153461753</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -1635,19 +1717,19 @@
         <v>170</v>
       </c>
       <c r="I20">
-        <v>0.9521889947121563</v>
+        <v>0.95218899471215634</v>
       </c>
       <c r="J20">
-        <v>0.931051288576299</v>
+        <v>0.93105128857629904</v>
       </c>
       <c r="K20">
-        <v>0.8616828951030119</v>
+        <v>0.86168289510301188</v>
       </c>
       <c r="L20">
-        <v>0.9274720459608826</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12">
+        <v>0.92747204596088262</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -1673,19 +1755,19 @@
         <v>170</v>
       </c>
       <c r="I21">
-        <v>0.9470596987118554</v>
+        <v>0.94705969871185536</v>
       </c>
       <c r="J21">
         <v>0.9143145472413764</v>
       </c>
       <c r="K21">
-        <v>0.7530451656901426</v>
+        <v>0.75304516569014257</v>
       </c>
       <c r="L21">
-        <v>0.8560410094499747</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12">
+        <v>0.85604100944997474</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -1711,19 +1793,19 @@
         <v>170</v>
       </c>
       <c r="I22">
-        <v>0.7133363542616962</v>
+        <v>0.71333635426169617</v>
       </c>
       <c r="J22">
-        <v>0.6619209039548022</v>
+        <v>0.66192090395480219</v>
       </c>
       <c r="K22">
         <v>0.7652941176470589</v>
       </c>
       <c r="L22">
-        <v>0.7252032520325203</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12">
+        <v>0.72520325203252034</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -1749,19 +1831,19 @@
         <v>170</v>
       </c>
       <c r="I23">
-        <v>0.7776691926403734</v>
+        <v>0.77766919264037337</v>
       </c>
       <c r="J23">
-        <v>0.7231317143630946</v>
+        <v>0.72313171436309465</v>
       </c>
       <c r="K23">
-        <v>0.7328798185941043</v>
+        <v>0.73287981859410434</v>
       </c>
       <c r="L23">
-        <v>0.7436314363143631</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12">
+        <v>0.74363143631436313</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -1787,19 +1869,19 @@
         <v>170</v>
       </c>
       <c r="I24">
-        <v>0.7459922539495089</v>
+        <v>0.74599225394950885</v>
       </c>
       <c r="J24">
         <v>0.6939572165971809</v>
       </c>
       <c r="K24">
-        <v>0.7069520070913005</v>
+        <v>0.70695200709130046</v>
       </c>
       <c r="L24">
-        <v>0.6850948509485095</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
+        <v>0.68509485094850953</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -1825,19 +1907,19 @@
         <v>170</v>
       </c>
       <c r="I25">
-        <v>0.7492074703191335</v>
+        <v>0.74920747031913348</v>
       </c>
       <c r="J25">
-        <v>0.694354920441877</v>
+        <v>0.69435492044187697</v>
       </c>
       <c r="K25">
-        <v>0.7449392712550608</v>
+        <v>0.74493927125506076</v>
       </c>
       <c r="L25">
-        <v>0.733739837398374</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12">
+        <v>0.73373983739837401</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -1863,19 +1945,19 @@
         <v>170</v>
       </c>
       <c r="I26">
-        <v>0.7392717478982493</v>
+        <v>0.73927174789824934</v>
       </c>
       <c r="J26">
-        <v>0.688479531840587</v>
+        <v>0.68847953184058697</v>
       </c>
       <c r="K26">
-        <v>0.7363758717729108</v>
+        <v>0.73637587177291075</v>
       </c>
       <c r="L26">
-        <v>0.7184281842818427</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12">
+        <v>0.71842818428184274</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -1901,19 +1983,19 @@
         <v>170</v>
       </c>
       <c r="I27">
-        <v>0.9599673571336063</v>
+        <v>0.95996735713360626</v>
       </c>
       <c r="J27">
-        <v>0.9594943240454075</v>
+        <v>0.95949432404540747</v>
       </c>
       <c r="K27">
-        <v>0.951575906889814</v>
+        <v>0.95157590688981397</v>
       </c>
       <c r="L27">
-        <v>0.9404761904761905</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12">
+        <v>0.94047619047619047</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -1939,19 +2021,19 @@
         <v>170</v>
       </c>
       <c r="I28">
-        <v>0.9684294999794067</v>
+        <v>0.96842949997940675</v>
       </c>
       <c r="J28">
-        <v>0.9661730647594025</v>
+        <v>0.96617306475940246</v>
       </c>
       <c r="K28">
-        <v>0.9521289997480473</v>
+        <v>0.95212899974804732</v>
       </c>
       <c r="L28">
-        <v>0.9454365079365079</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12">
+        <v>0.94543650793650791</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -1977,19 +2059,19 @@
         <v>170</v>
       </c>
       <c r="I29">
-        <v>0.9570400941270751</v>
+        <v>0.95704009412707514</v>
       </c>
       <c r="J29">
-        <v>0.9550363207483951</v>
+        <v>0.95503632074839506</v>
       </c>
       <c r="K29">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L29">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -2015,19 +2097,19 @@
         <v>170</v>
       </c>
       <c r="I30">
-        <v>0.9560568916037298</v>
+        <v>0.95605689160372975</v>
       </c>
       <c r="J30">
-        <v>0.9537824675324676</v>
+        <v>0.95378246753246765</v>
       </c>
       <c r="K30">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L30">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -2056,16 +2138,16 @@
         <v>0.9599558564761661</v>
       </c>
       <c r="J31">
-        <v>0.9577335858585858</v>
+        <v>0.95773358585858581</v>
       </c>
       <c r="K31">
-        <v>0.9521289997480473</v>
+        <v>0.95212899974804732</v>
       </c>
       <c r="L31">
-        <v>0.9454365079365079</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12">
+        <v>0.94543650793650791</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -2088,19 +2170,19 @@
         <v>418</v>
       </c>
       <c r="I32">
-        <v>0.8954576367301528</v>
+        <v>0.89545763673015277</v>
       </c>
       <c r="J32">
-        <v>0.8970525030525029</v>
+        <v>0.89705250305250295</v>
       </c>
       <c r="K32">
-        <v>0.2667521367521367</v>
+        <v>0.26675213675213671</v>
       </c>
       <c r="L32">
-        <v>0.2813852813852813</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12">
+        <v>0.28138528138528129</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -2123,19 +2205,19 @@
         <v>379</v>
       </c>
       <c r="I33">
-        <v>0.9195943125759042</v>
+        <v>0.91959431257590418</v>
       </c>
       <c r="J33">
-        <v>0.9206028985507247</v>
+        <v>0.92060289855072475</v>
       </c>
       <c r="K33">
-        <v>0.2780092592592592</v>
+        <v>0.27800925925925918</v>
       </c>
       <c r="L33">
-        <v>0.2935064935064935</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12">
+        <v>0.29350649350649349</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>13</v>
       </c>
@@ -2161,16 +2243,16 @@
         <v>0.9078352154149838</v>
       </c>
       <c r="J34">
-        <v>0.9090259666259666</v>
+        <v>0.90902596662596657</v>
       </c>
       <c r="K34">
-        <v>0.2320375106564365</v>
+        <v>0.23203751065643649</v>
       </c>
       <c r="L34">
-        <v>0.2406926406926407</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12">
+        <v>0.24069264069264071</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>13</v>
       </c>
@@ -2193,19 +2275,19 @@
         <v>400</v>
       </c>
       <c r="I35">
-        <v>0.8928899485383743</v>
+        <v>0.89288994853837433</v>
       </c>
       <c r="J35">
-        <v>0.8938649572649572</v>
+        <v>0.89386495726495718</v>
       </c>
       <c r="K35">
-        <v>0.2723076923076923</v>
+        <v>0.27230769230769231</v>
       </c>
       <c r="L35">
-        <v>0.2891774891774891</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12">
+        <v>0.28917748917748909</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>13</v>
       </c>
@@ -2228,19 +2310,19 @@
         <v>401</v>
       </c>
       <c r="I36">
-        <v>0.9153934258621577</v>
+        <v>0.91539342586215766</v>
       </c>
       <c r="J36">
-        <v>0.9164136752136752</v>
+        <v>0.91641367521367523</v>
       </c>
       <c r="K36">
-        <v>0.3015705128205128</v>
+        <v>0.30157051282051278</v>
       </c>
       <c r="L36">
-        <v>0.3038961038961038</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12">
+        <v>0.30389610389610378</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>13</v>
       </c>
@@ -2263,19 +2345,19 @@
         <v>208961</v>
       </c>
       <c r="I37">
-        <v>0.9999490830944178</v>
+        <v>0.99994908309441777</v>
       </c>
       <c r="J37">
-        <v>0.9999490779492387</v>
+        <v>0.99994907794923871</v>
       </c>
       <c r="K37">
-        <v>0.95227165081794</v>
+        <v>0.95227165081793996</v>
       </c>
       <c r="L37">
         <v>0.9285714285714286</v>
       </c>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -2298,27 +2380,27 @@
         <v>187962</v>
       </c>
       <c r="I38">
-        <v>0.9999695295796485</v>
+        <v>0.99996952957964846</v>
       </c>
       <c r="J38">
-        <v>0.9999695326305527</v>
+        <v>0.99996953263055266</v>
       </c>
       <c r="K38">
-        <v>0.9446616556880125</v>
+        <v>0.94466165568801252</v>
       </c>
       <c r="L38">
-        <v>0.9995737980278344</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12">
+        <v>0.99957379802783441</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B39" t="s">
         <v>20</v>
       </c>
       <c r="C39" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="D39">
         <v>57532</v>
@@ -2330,13 +2412,13 @@
         <v>45932</v>
       </c>
       <c r="H39">
-        <v>206831</v>
+        <v>170731</v>
       </c>
       <c r="I39">
-        <v>0.9999683427841612</v>
+        <v>0.99996834278416125</v>
       </c>
       <c r="J39">
-        <v>0.9999683454148334</v>
+        <v>0.99996834541483337</v>
       </c>
       <c r="K39">
         <v>1</v>
@@ -2345,7 +2427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -2368,19 +2450,19 @@
         <v>202727</v>
       </c>
       <c r="I40">
-        <v>0.9999838482536472</v>
+        <v>0.99998384825364717</v>
       </c>
       <c r="J40">
-        <v>0.9999838460855026</v>
+        <v>0.99998384608550261</v>
       </c>
       <c r="K40">
-        <v>0.9487925934843959</v>
+        <v>0.94879259348439593</v>
       </c>
       <c r="L40">
-        <v>0.99968534841644</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12">
+        <v>0.99968534841643997</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -2403,19 +2485,19 @@
         <v>198466</v>
       </c>
       <c r="I41">
-        <v>0.9999752606897528</v>
+        <v>0.99997526068975284</v>
       </c>
       <c r="J41">
-        <v>0.9999752590242525</v>
+        <v>0.99997525902425255</v>
       </c>
       <c r="K41">
-        <v>0.9774734911308108</v>
+        <v>0.97747349113081083</v>
       </c>
       <c r="L41">
-        <v>0.9999041189261753</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12">
+        <v>0.99990411892617526</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -2438,19 +2520,19 @@
         <v>1368</v>
       </c>
       <c r="I42">
-        <v>0.9696022159390552</v>
+        <v>0.96960221593905516</v>
       </c>
       <c r="J42">
-        <v>0.9695222616335117</v>
+        <v>0.96952226163351174</v>
       </c>
       <c r="K42">
-        <v>0.7588638195004029</v>
+        <v>0.75886381950040294</v>
       </c>
       <c r="L42">
-        <v>0.7909214092140922</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12">
+        <v>0.79092140921409215</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -2473,19 +2555,19 @@
         <v>1247</v>
       </c>
       <c r="I43">
-        <v>0.9720128069125031</v>
+        <v>0.97201280691250314</v>
       </c>
       <c r="J43">
-        <v>0.9718549594064534</v>
+        <v>0.97185495940645339</v>
       </c>
       <c r="K43">
-        <v>0.731894878303718</v>
+        <v>0.73189487830371802</v>
       </c>
       <c r="L43">
         <v>0.7827913279132791</v>
       </c>
     </row>
-    <row r="44" spans="1:12">
+    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -2508,19 +2590,19 @@
         <v>1342</v>
       </c>
       <c r="I44">
-        <v>0.9708745467525655</v>
+        <v>0.97087454675256546</v>
       </c>
       <c r="J44">
-        <v>0.970890410958904</v>
+        <v>0.97089041095890405</v>
       </c>
       <c r="K44">
-        <v>0.7068947423654108</v>
+        <v>0.70689474236541083</v>
       </c>
       <c r="L44">
-        <v>0.72289972899729</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12">
+        <v>0.72289972899729005</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -2546,16 +2628,16 @@
         <v>0.9680525004256525</v>
       </c>
       <c r="J45">
-        <v>0.9681498079385402</v>
+        <v>0.96814980793854022</v>
       </c>
       <c r="K45">
-        <v>0.7382358203614243</v>
+        <v>0.73823582036142432</v>
       </c>
       <c r="L45">
-        <v>0.7715447154471544</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12">
+        <v>0.77154471544715442</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -2581,16 +2663,16 @@
         <v>0.9697877581273302</v>
       </c>
       <c r="J46">
-        <v>0.9699646706895662</v>
+        <v>0.96996467068956616</v>
       </c>
       <c r="K46">
-        <v>0.7382358203614243</v>
+        <v>0.73823582036142432</v>
       </c>
       <c r="L46">
-        <v>0.7715447154471544</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12">
+        <v>0.77154471544715442</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -2613,19 +2695,19 @@
         <v>121</v>
       </c>
       <c r="I47">
-        <v>0.970437467848269</v>
+        <v>0.97043746784826901</v>
       </c>
       <c r="J47">
-        <v>0.9702661826981245</v>
+        <v>0.97026618269812448</v>
       </c>
       <c r="K47">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L47">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="48" spans="1:12">
+    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -2648,19 +2730,19 @@
         <v>101</v>
       </c>
       <c r="I48">
-        <v>0.9862724360605457</v>
+        <v>0.98627243606054571</v>
       </c>
       <c r="J48">
-        <v>0.9863499245852188</v>
+        <v>0.98634992458521875</v>
       </c>
       <c r="K48">
-        <v>0.9619111259605747</v>
+        <v>0.96191112596057471</v>
       </c>
       <c r="L48">
-        <v>0.9573412698412699</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12">
+        <v>0.95734126984126988</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -2683,19 +2765,19 @@
         <v>121</v>
       </c>
       <c r="I49">
-        <v>0.9702280024393483</v>
+        <v>0.97022800243934826</v>
       </c>
       <c r="J49">
-        <v>0.9700760521994642</v>
+        <v>0.97007605219946424</v>
       </c>
       <c r="K49">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L49">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="50" spans="1:12">
+    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>13</v>
       </c>
@@ -2718,19 +2800,19 @@
         <v>115</v>
       </c>
       <c r="I50">
-        <v>0.9783695982380193</v>
+        <v>0.97836959823801928</v>
       </c>
       <c r="J50">
         <v>0.9783441558441559</v>
       </c>
       <c r="K50">
-        <v>0.9811507936507937</v>
+        <v>0.98115079365079372</v>
       </c>
       <c r="L50">
-        <v>0.9811507936507937</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12">
+        <v>0.98115079365079372</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -2753,19 +2835,19 @@
         <v>111</v>
       </c>
       <c r="I51">
-        <v>0.9722986539544465</v>
+        <v>0.97229865395444648</v>
       </c>
       <c r="J51">
         <v>0.9722895622895622</v>
       </c>
       <c r="K51">
-        <v>0.9715828832571667</v>
+        <v>0.97158288325716669</v>
       </c>
       <c r="L51">
-        <v>0.9692460317460317</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12">
+        <v>0.96924603174603174</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>14</v>
       </c>
@@ -2788,19 +2870,19 @@
         <v>195</v>
       </c>
       <c r="I52">
-        <v>0.9203058592248997</v>
+        <v>0.92030585922489971</v>
       </c>
       <c r="J52">
-        <v>0.9220085470085471</v>
+        <v>0.92200854700854706</v>
       </c>
       <c r="K52">
-        <v>0.789751552795031</v>
+        <v>0.78975155279503095</v>
       </c>
       <c r="L52">
-        <v>0.8841269841269841</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12">
+        <v>0.88412698412698409</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>14</v>
       </c>
@@ -2823,19 +2905,19 @@
         <v>142</v>
       </c>
       <c r="I53">
-        <v>0.9026875628820707</v>
+        <v>0.90268756288207075</v>
       </c>
       <c r="J53">
         <v>0.9015151515151516</v>
       </c>
       <c r="K53">
-        <v>0.7216738816738816</v>
+        <v>0.72167388167388158</v>
       </c>
       <c r="L53">
-        <v>0.7896825396825397</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12">
+        <v>0.78968253968253965</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>14</v>
       </c>
@@ -2858,19 +2940,19 @@
         <v>194</v>
       </c>
       <c r="I54">
-        <v>0.9086135667874797</v>
+        <v>0.90861356678747973</v>
       </c>
       <c r="J54">
-        <v>0.913888888888889</v>
+        <v>0.91388888888888897</v>
       </c>
       <c r="K54">
-        <v>0.8099206349206348</v>
+        <v>0.80992063492063482</v>
       </c>
       <c r="L54">
-        <v>0.8960317460317461</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12">
+        <v>0.89603174603174607</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>14</v>
       </c>
@@ -2896,16 +2978,16 @@
         <v>0.9002709555608106</v>
       </c>
       <c r="J55">
-        <v>0.9020202020202021</v>
+        <v>0.90202020202020206</v>
       </c>
       <c r="K55">
-        <v>0.7774250440917108</v>
+        <v>0.77742504409171076</v>
       </c>
       <c r="L55">
-        <v>0.873015873015873</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12">
+        <v>0.87301587301587302</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>14</v>
       </c>
@@ -2931,16 +3013,16 @@
         <v>0.9135364394060046</v>
       </c>
       <c r="J56">
-        <v>0.9154040404040404</v>
+        <v>0.91540404040404044</v>
       </c>
       <c r="K56">
-        <v>0.7764367816091954</v>
+        <v>0.77643678160919538</v>
       </c>
       <c r="L56">
         <v>0.8563492063492063</v>
       </c>
     </row>
-    <row r="57" spans="1:12">
+    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>14</v>
       </c>
@@ -2963,19 +3045,19 @@
         <v>413</v>
       </c>
       <c r="I57">
-        <v>0.8954576367301528</v>
+        <v>0.89545763673015277</v>
       </c>
       <c r="J57">
-        <v>0.8970525030525029</v>
+        <v>0.89705250305250295</v>
       </c>
       <c r="K57">
-        <v>0.2667521367521367</v>
+        <v>0.26675213675213671</v>
       </c>
       <c r="L57">
-        <v>0.2813852813852813</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12">
+        <v>0.28138528138528129</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -2998,19 +3080,19 @@
         <v>373</v>
       </c>
       <c r="I58">
-        <v>0.9195943125759042</v>
+        <v>0.91959431257590418</v>
       </c>
       <c r="J58">
-        <v>0.9206028985507247</v>
+        <v>0.92060289855072475</v>
       </c>
       <c r="K58">
-        <v>0.2780092592592592</v>
+        <v>0.27800925925925918</v>
       </c>
       <c r="L58">
-        <v>0.2935064935064935</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12">
+        <v>0.29350649350649349</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>14</v>
       </c>
@@ -3036,16 +3118,16 @@
         <v>0.9078352154149838</v>
       </c>
       <c r="J59">
-        <v>0.9090259666259666</v>
+        <v>0.90902596662596657</v>
       </c>
       <c r="K59">
-        <v>0.2320375106564365</v>
+        <v>0.23203751065643649</v>
       </c>
       <c r="L59">
-        <v>0.2406926406926407</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12">
+        <v>0.24069264069264071</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>14</v>
       </c>
@@ -3068,19 +3150,19 @@
         <v>402</v>
       </c>
       <c r="I60">
-        <v>0.8928899485383743</v>
+        <v>0.89288994853837433</v>
       </c>
       <c r="J60">
-        <v>0.8938649572649572</v>
+        <v>0.89386495726495718</v>
       </c>
       <c r="K60">
-        <v>0.2723076923076923</v>
+        <v>0.27230769230769231</v>
       </c>
       <c r="L60">
-        <v>0.2891774891774891</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12">
+        <v>0.28917748917748909</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>14</v>
       </c>
@@ -3103,19 +3185,19 @@
         <v>393</v>
       </c>
       <c r="I61">
-        <v>0.9153934258621577</v>
+        <v>0.91539342586215766</v>
       </c>
       <c r="J61">
-        <v>0.9164136752136752</v>
+        <v>0.91641367521367523</v>
       </c>
       <c r="K61">
-        <v>0.3015705128205128</v>
+        <v>0.30157051282051278</v>
       </c>
       <c r="L61">
-        <v>0.3038961038961038</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12">
+        <v>0.30389610389610378</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>14</v>
       </c>
@@ -3138,19 +3220,19 @@
         <v>172454</v>
       </c>
       <c r="I62">
-        <v>0.9999490830944178</v>
+        <v>0.99994908309441777</v>
       </c>
       <c r="J62">
-        <v>0.9999490779492387</v>
+        <v>0.99994907794923871</v>
       </c>
       <c r="K62">
-        <v>0.95227165081794</v>
+        <v>0.95227165081793996</v>
       </c>
       <c r="L62">
         <v>0.9285714285714286</v>
       </c>
     </row>
-    <row r="63" spans="1:12">
+    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>14</v>
       </c>
@@ -3173,27 +3255,27 @@
         <v>155209</v>
       </c>
       <c r="I63">
-        <v>0.9999695295796485</v>
+        <v>0.99996952957964846</v>
       </c>
       <c r="J63">
-        <v>0.9999695326305527</v>
+        <v>0.99996953263055266</v>
       </c>
       <c r="K63">
-        <v>0.9446616556880125</v>
+        <v>0.94466165568801252</v>
       </c>
       <c r="L63">
-        <v>0.9995737980278344</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12">
+        <v>0.99957379802783441</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B64" t="s">
         <v>20</v>
       </c>
       <c r="C64" t="s">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="D64">
         <v>57532</v>
@@ -3205,13 +3287,13 @@
         <v>45932</v>
       </c>
       <c r="H64">
-        <v>170731</v>
+        <v>206796</v>
       </c>
       <c r="I64">
-        <v>0.9999683427841612</v>
+        <v>0.99996834278416125</v>
       </c>
       <c r="J64">
-        <v>0.9999683454148334</v>
+        <v>0.99996834541483337</v>
       </c>
       <c r="K64">
         <v>1</v>
@@ -3220,7 +3302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>14</v>
       </c>
@@ -3243,19 +3325,19 @@
         <v>167277</v>
       </c>
       <c r="I65">
-        <v>0.9999838482536472</v>
+        <v>0.99998384825364717</v>
       </c>
       <c r="J65">
-        <v>0.9999838460855026</v>
+        <v>0.99998384608550261</v>
       </c>
       <c r="K65">
-        <v>0.9487925934843959</v>
+        <v>0.94879259348439593</v>
       </c>
       <c r="L65">
-        <v>0.99968534841644</v>
-      </c>
-    </row>
-    <row r="66" spans="1:12">
+        <v>0.99968534841643997</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>14</v>
       </c>
@@ -3278,19 +3360,19 @@
         <v>163830</v>
       </c>
       <c r="I66">
-        <v>0.9999752606897528</v>
+        <v>0.99997526068975284</v>
       </c>
       <c r="J66">
-        <v>0.9999752590242525</v>
+        <v>0.99997525902425255</v>
       </c>
       <c r="K66">
-        <v>0.9774734911308108</v>
+        <v>0.97747349113081083</v>
       </c>
       <c r="L66">
-        <v>0.9999041189261753</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12">
+        <v>0.99990411892617526</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>14</v>
       </c>
@@ -3313,19 +3395,19 @@
         <v>1355</v>
       </c>
       <c r="I67">
-        <v>0.9696022159390552</v>
+        <v>0.96960221593905516</v>
       </c>
       <c r="J67">
-        <v>0.9695222616335117</v>
+        <v>0.96952226163351174</v>
       </c>
       <c r="K67">
-        <v>0.7588638195004029</v>
+        <v>0.75886381950040294</v>
       </c>
       <c r="L67">
-        <v>0.7909214092140922</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12">
+        <v>0.79092140921409215</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>14</v>
       </c>
@@ -3348,19 +3430,19 @@
         <v>1219</v>
       </c>
       <c r="I68">
-        <v>0.9720128069125031</v>
+        <v>0.97201280691250314</v>
       </c>
       <c r="J68">
-        <v>0.9718549594064534</v>
+        <v>0.97185495940645339</v>
       </c>
       <c r="K68">
-        <v>0.731894878303718</v>
+        <v>0.73189487830371802</v>
       </c>
       <c r="L68">
         <v>0.7827913279132791</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>14</v>
       </c>
@@ -3383,19 +3465,19 @@
         <v>1342</v>
       </c>
       <c r="I69">
-        <v>0.9708745467525655</v>
+        <v>0.97087454675256546</v>
       </c>
       <c r="J69">
-        <v>0.970890410958904</v>
+        <v>0.97089041095890405</v>
       </c>
       <c r="K69">
-        <v>0.7068947423654108</v>
+        <v>0.70689474236541083</v>
       </c>
       <c r="L69">
-        <v>0.72289972899729</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12">
+        <v>0.72289972899729005</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>14</v>
       </c>
@@ -3421,16 +3503,16 @@
         <v>0.9680525004256525</v>
       </c>
       <c r="J70">
-        <v>0.9681498079385402</v>
+        <v>0.96814980793854022</v>
       </c>
       <c r="K70">
-        <v>0.7382358203614243</v>
+        <v>0.73823582036142432</v>
       </c>
       <c r="L70">
-        <v>0.7715447154471544</v>
-      </c>
-    </row>
-    <row r="71" spans="1:12">
+        <v>0.77154471544715442</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>14</v>
       </c>
@@ -3456,16 +3538,16 @@
         <v>0.9697877581273302</v>
       </c>
       <c r="J71">
-        <v>0.9699646706895662</v>
+        <v>0.96996467068956616</v>
       </c>
       <c r="K71">
-        <v>0.7382358203614243</v>
+        <v>0.73823582036142432</v>
       </c>
       <c r="L71">
-        <v>0.7715447154471544</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12">
+        <v>0.77154471544715442</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>14</v>
       </c>
@@ -3488,19 +3570,19 @@
         <v>115</v>
       </c>
       <c r="I72">
-        <v>0.970437467848269</v>
+        <v>0.97043746784826901</v>
       </c>
       <c r="J72">
-        <v>0.9702661826981245</v>
+        <v>0.97026618269812448</v>
       </c>
       <c r="K72">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L72">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>14</v>
       </c>
@@ -3523,19 +3605,19 @@
         <v>103</v>
       </c>
       <c r="I73">
-        <v>0.9862724360605457</v>
+        <v>0.98627243606054571</v>
       </c>
       <c r="J73">
-        <v>0.9863499245852188</v>
+        <v>0.98634992458521875</v>
       </c>
       <c r="K73">
-        <v>0.9619111259605747</v>
+        <v>0.96191112596057471</v>
       </c>
       <c r="L73">
-        <v>0.9573412698412699</v>
-      </c>
-    </row>
-    <row r="74" spans="1:12">
+        <v>0.95734126984126988</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>14</v>
       </c>
@@ -3558,19 +3640,19 @@
         <v>114</v>
       </c>
       <c r="I74">
-        <v>0.9702280024393483</v>
+        <v>0.97022800243934826</v>
       </c>
       <c r="J74">
-        <v>0.9700760521994642</v>
+        <v>0.97007605219946424</v>
       </c>
       <c r="K74">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L74">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>14</v>
       </c>
@@ -3593,19 +3675,19 @@
         <v>112</v>
       </c>
       <c r="I75">
-        <v>0.9783695982380193</v>
+        <v>0.97836959823801928</v>
       </c>
       <c r="J75">
         <v>0.9783441558441559</v>
       </c>
       <c r="K75">
-        <v>0.9811507936507937</v>
+        <v>0.98115079365079372</v>
       </c>
       <c r="L75">
-        <v>0.9811507936507937</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12">
+        <v>0.98115079365079372</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -3628,19 +3710,19 @@
         <v>109</v>
       </c>
       <c r="I76">
-        <v>0.9722986539544465</v>
+        <v>0.97229865395444648</v>
       </c>
       <c r="J76">
         <v>0.9722895622895622</v>
       </c>
       <c r="K76">
-        <v>0.9715828832571667</v>
+        <v>0.97158288325716669</v>
       </c>
       <c r="L76">
-        <v>0.9692460317460317</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12">
+        <v>0.96924603174603174</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>15</v>
       </c>
@@ -3663,19 +3745,19 @@
         <v>195</v>
       </c>
       <c r="I77">
-        <v>0.9203058592248997</v>
+        <v>0.92030585922489971</v>
       </c>
       <c r="J77">
-        <v>0.9220085470085471</v>
+        <v>0.92200854700854706</v>
       </c>
       <c r="K77">
-        <v>0.789751552795031</v>
+        <v>0.78975155279503095</v>
       </c>
       <c r="L77">
-        <v>0.8841269841269841</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12">
+        <v>0.88412698412698409</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>15</v>
       </c>
@@ -3698,19 +3780,19 @@
         <v>177</v>
       </c>
       <c r="I78">
-        <v>0.9026875628820707</v>
+        <v>0.90268756288207075</v>
       </c>
       <c r="J78">
         <v>0.9015151515151516</v>
       </c>
       <c r="K78">
-        <v>0.7216738816738816</v>
+        <v>0.72167388167388158</v>
       </c>
       <c r="L78">
-        <v>0.7896825396825397</v>
-      </c>
-    </row>
-    <row r="79" spans="1:12">
+        <v>0.78968253968253965</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>15</v>
       </c>
@@ -3733,19 +3815,19 @@
         <v>194</v>
       </c>
       <c r="I79">
-        <v>0.9086135667874797</v>
+        <v>0.90861356678747973</v>
       </c>
       <c r="J79">
-        <v>0.913888888888889</v>
+        <v>0.91388888888888897</v>
       </c>
       <c r="K79">
-        <v>0.8099206349206348</v>
+        <v>0.80992063492063482</v>
       </c>
       <c r="L79">
-        <v>0.8960317460317461</v>
-      </c>
-    </row>
-    <row r="80" spans="1:12">
+        <v>0.89603174603174607</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>15</v>
       </c>
@@ -3771,16 +3853,16 @@
         <v>0.9002709555608106</v>
       </c>
       <c r="J80">
-        <v>0.9020202020202021</v>
+        <v>0.90202020202020206</v>
       </c>
       <c r="K80">
-        <v>0.7774250440917108</v>
+        <v>0.77742504409171076</v>
       </c>
       <c r="L80">
-        <v>0.873015873015873</v>
-      </c>
-    </row>
-    <row r="81" spans="1:12">
+        <v>0.87301587301587302</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>15</v>
       </c>
@@ -3806,16 +3888,16 @@
         <v>0.9135364394060046</v>
       </c>
       <c r="J81">
-        <v>0.9154040404040404</v>
+        <v>0.91540404040404044</v>
       </c>
       <c r="K81">
-        <v>0.7764367816091954</v>
+        <v>0.77643678160919538</v>
       </c>
       <c r="L81">
         <v>0.8563492063492063</v>
       </c>
     </row>
-    <row r="82" spans="1:12">
+    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>15</v>
       </c>
@@ -3838,19 +3920,19 @@
         <v>413</v>
       </c>
       <c r="I82">
-        <v>0.8954576367301528</v>
+        <v>0.89545763673015277</v>
       </c>
       <c r="J82">
-        <v>0.8970525030525029</v>
+        <v>0.89705250305250295</v>
       </c>
       <c r="K82">
-        <v>0.2667521367521367</v>
+        <v>0.26675213675213671</v>
       </c>
       <c r="L82">
-        <v>0.2813852813852813</v>
-      </c>
-    </row>
-    <row r="83" spans="1:12">
+        <v>0.28138528138528129</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>15</v>
       </c>
@@ -3873,19 +3955,19 @@
         <v>373</v>
       </c>
       <c r="I83">
-        <v>0.9195943125759042</v>
+        <v>0.91959431257590418</v>
       </c>
       <c r="J83">
-        <v>0.9206028985507247</v>
+        <v>0.92060289855072475</v>
       </c>
       <c r="K83">
-        <v>0.2780092592592592</v>
+        <v>0.27800925925925918</v>
       </c>
       <c r="L83">
-        <v>0.2935064935064935</v>
-      </c>
-    </row>
-    <row r="84" spans="1:12">
+        <v>0.29350649350649349</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>15</v>
       </c>
@@ -3911,16 +3993,16 @@
         <v>0.9078352154149838</v>
       </c>
       <c r="J84">
-        <v>0.9090259666259666</v>
+        <v>0.90902596662596657</v>
       </c>
       <c r="K84">
-        <v>0.2320375106564365</v>
+        <v>0.23203751065643649</v>
       </c>
       <c r="L84">
-        <v>0.2406926406926407</v>
-      </c>
-    </row>
-    <row r="85" spans="1:12">
+        <v>0.24069264069264071</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>15</v>
       </c>
@@ -3943,19 +4025,19 @@
         <v>402</v>
       </c>
       <c r="I85">
-        <v>0.8928899485383743</v>
+        <v>0.89288994853837433</v>
       </c>
       <c r="J85">
-        <v>0.8938649572649572</v>
+        <v>0.89386495726495718</v>
       </c>
       <c r="K85">
-        <v>0.2723076923076923</v>
+        <v>0.27230769230769231</v>
       </c>
       <c r="L85">
-        <v>0.2891774891774891</v>
-      </c>
-    </row>
-    <row r="86" spans="1:12">
+        <v>0.28917748917748909</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>15</v>
       </c>
@@ -3978,19 +4060,19 @@
         <v>393</v>
       </c>
       <c r="I86">
-        <v>0.9153934258621577</v>
+        <v>0.91539342586215766</v>
       </c>
       <c r="J86">
-        <v>0.9164136752136752</v>
+        <v>0.91641367521367523</v>
       </c>
       <c r="K86">
-        <v>0.3015705128205128</v>
+        <v>0.30157051282051278</v>
       </c>
       <c r="L86">
-        <v>0.3038961038961038</v>
-      </c>
-    </row>
-    <row r="87" spans="1:12">
+        <v>0.30389610389610378</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>15</v>
       </c>
@@ -4013,19 +4095,19 @@
         <v>208883</v>
       </c>
       <c r="I87">
-        <v>0.9999490830944178</v>
+        <v>0.99994908309441777</v>
       </c>
       <c r="J87">
-        <v>0.9999490779492387</v>
+        <v>0.99994907794923871</v>
       </c>
       <c r="K87">
-        <v>0.95227165081794</v>
+        <v>0.95227165081793996</v>
       </c>
       <c r="L87">
         <v>0.9285714285714286</v>
       </c>
     </row>
-    <row r="88" spans="1:12">
+    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>15</v>
       </c>
@@ -4048,27 +4130,27 @@
         <v>187995</v>
       </c>
       <c r="I88">
-        <v>0.9999695295796485</v>
+        <v>0.99996952957964846</v>
       </c>
       <c r="J88">
-        <v>0.9999695326305527</v>
+        <v>0.99996953263055266</v>
       </c>
       <c r="K88">
-        <v>0.9446616556880125</v>
+        <v>0.94466165568801252</v>
       </c>
       <c r="L88">
-        <v>0.9995737980278344</v>
-      </c>
-    </row>
-    <row r="89" spans="1:12">
+        <v>0.99957379802783441</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B89" t="s">
         <v>20</v>
       </c>
       <c r="C89" t="s">
-        <v>110</v>
+        <v>155</v>
       </c>
       <c r="D89">
         <v>57532</v>
@@ -4079,23 +4161,26 @@
       <c r="F89">
         <v>45932</v>
       </c>
+      <c r="G89">
+        <v>2728</v>
+      </c>
       <c r="H89">
-        <v>206796</v>
+        <v>170700</v>
       </c>
       <c r="I89">
-        <v>0.9999683427841612</v>
+        <v>0.96595276227314386</v>
       </c>
       <c r="J89">
-        <v>0.9999683454148334</v>
+        <v>0.94640087366655057</v>
       </c>
       <c r="K89">
-        <v>1</v>
+        <v>0.85699346095653384</v>
       </c>
       <c r="L89">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:12">
+        <v>0.8571428571428571</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>15</v>
       </c>
@@ -4118,19 +4203,19 @@
         <v>202613</v>
       </c>
       <c r="I90">
-        <v>0.9999838482536472</v>
+        <v>0.99998384825364717</v>
       </c>
       <c r="J90">
-        <v>0.9999838460855026</v>
+        <v>0.99998384608550261</v>
       </c>
       <c r="K90">
-        <v>0.9487925934843959</v>
+        <v>0.94879259348439593</v>
       </c>
       <c r="L90">
-        <v>0.99968534841644</v>
-      </c>
-    </row>
-    <row r="91" spans="1:12">
+        <v>0.99968534841643997</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>15</v>
       </c>
@@ -4153,19 +4238,19 @@
         <v>198437</v>
       </c>
       <c r="I91">
-        <v>0.9999752606897528</v>
+        <v>0.99997526068975284</v>
       </c>
       <c r="J91">
-        <v>0.9999752590242525</v>
+        <v>0.99997525902425255</v>
       </c>
       <c r="K91">
-        <v>0.9774734911308108</v>
+        <v>0.97747349113081083</v>
       </c>
       <c r="L91">
-        <v>0.9999041189261753</v>
-      </c>
-    </row>
-    <row r="92" spans="1:12">
+        <v>0.99990411892617526</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>15</v>
       </c>
@@ -4188,19 +4273,19 @@
         <v>1355</v>
       </c>
       <c r="I92">
-        <v>0.9696022159390552</v>
+        <v>0.96960221593905516</v>
       </c>
       <c r="J92">
-        <v>0.9695222616335117</v>
+        <v>0.96952226163351174</v>
       </c>
       <c r="K92">
-        <v>0.7588638195004029</v>
+        <v>0.75886381950040294</v>
       </c>
       <c r="L92">
-        <v>0.7909214092140922</v>
-      </c>
-    </row>
-    <row r="93" spans="1:12">
+        <v>0.79092140921409215</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>15</v>
       </c>
@@ -4223,19 +4308,19 @@
         <v>1219</v>
       </c>
       <c r="I93">
-        <v>0.9720128069125031</v>
+        <v>0.97201280691250314</v>
       </c>
       <c r="J93">
-        <v>0.9718549594064534</v>
+        <v>0.97185495940645339</v>
       </c>
       <c r="K93">
-        <v>0.731894878303718</v>
+        <v>0.73189487830371802</v>
       </c>
       <c r="L93">
         <v>0.7827913279132791</v>
       </c>
     </row>
-    <row r="94" spans="1:12">
+    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>15</v>
       </c>
@@ -4258,19 +4343,19 @@
         <v>1342</v>
       </c>
       <c r="I94">
-        <v>0.9708745467525655</v>
+        <v>0.97087454675256546</v>
       </c>
       <c r="J94">
-        <v>0.970890410958904</v>
+        <v>0.97089041095890405</v>
       </c>
       <c r="K94">
-        <v>0.7068947423654108</v>
+        <v>0.70689474236541083</v>
       </c>
       <c r="L94">
-        <v>0.72289972899729</v>
-      </c>
-    </row>
-    <row r="95" spans="1:12">
+        <v>0.72289972899729005</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>15</v>
       </c>
@@ -4296,16 +4381,16 @@
         <v>0.9680525004256525</v>
       </c>
       <c r="J95">
-        <v>0.9681498079385402</v>
+        <v>0.96814980793854022</v>
       </c>
       <c r="K95">
-        <v>0.7382358203614243</v>
+        <v>0.73823582036142432</v>
       </c>
       <c r="L95">
-        <v>0.7715447154471544</v>
-      </c>
-    </row>
-    <row r="96" spans="1:12">
+        <v>0.77154471544715442</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>15</v>
       </c>
@@ -4331,16 +4416,16 @@
         <v>0.9697877581273302</v>
       </c>
       <c r="J96">
-        <v>0.9699646706895662</v>
+        <v>0.96996467068956616</v>
       </c>
       <c r="K96">
-        <v>0.7382358203614243</v>
+        <v>0.73823582036142432</v>
       </c>
       <c r="L96">
-        <v>0.7715447154471544</v>
-      </c>
-    </row>
-    <row r="97" spans="1:12">
+        <v>0.77154471544715442</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>15</v>
       </c>
@@ -4363,19 +4448,19 @@
         <v>115</v>
       </c>
       <c r="I97">
-        <v>0.970437467848269</v>
+        <v>0.97043746784826901</v>
       </c>
       <c r="J97">
-        <v>0.9702661826981245</v>
+        <v>0.97026618269812448</v>
       </c>
       <c r="K97">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L97">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="98" spans="1:12">
+    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>15</v>
       </c>
@@ -4398,19 +4483,19 @@
         <v>103</v>
       </c>
       <c r="I98">
-        <v>0.9862724360605457</v>
+        <v>0.98627243606054571</v>
       </c>
       <c r="J98">
-        <v>0.9863499245852188</v>
+        <v>0.98634992458521875</v>
       </c>
       <c r="K98">
-        <v>0.9619111259605747</v>
+        <v>0.96191112596057471</v>
       </c>
       <c r="L98">
-        <v>0.9573412698412699</v>
-      </c>
-    </row>
-    <row r="99" spans="1:12">
+        <v>0.95734126984126988</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>15</v>
       </c>
@@ -4433,19 +4518,19 @@
         <v>114</v>
       </c>
       <c r="I99">
-        <v>0.9702280024393483</v>
+        <v>0.97022800243934826</v>
       </c>
       <c r="J99">
-        <v>0.9700760521994642</v>
+        <v>0.97007605219946424</v>
       </c>
       <c r="K99">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L99">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="100" spans="1:12">
+    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>15</v>
       </c>
@@ -4468,19 +4553,19 @@
         <v>112</v>
       </c>
       <c r="I100">
-        <v>0.9783695982380193</v>
+        <v>0.97836959823801928</v>
       </c>
       <c r="J100">
         <v>0.9783441558441559</v>
       </c>
       <c r="K100">
-        <v>0.9811507936507937</v>
+        <v>0.98115079365079372</v>
       </c>
       <c r="L100">
-        <v>0.9811507936507937</v>
-      </c>
-    </row>
-    <row r="101" spans="1:12">
+        <v>0.98115079365079372</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>15</v>
       </c>
@@ -4503,19 +4588,19 @@
         <v>109</v>
       </c>
       <c r="I101">
-        <v>0.9722986539544465</v>
+        <v>0.97229865395444648</v>
       </c>
       <c r="J101">
         <v>0.9722895622895622</v>
       </c>
       <c r="K101">
-        <v>0.9715828832571667</v>
+        <v>0.97158288325716669</v>
       </c>
       <c r="L101">
-        <v>0.9692460317460317</v>
-      </c>
-    </row>
-    <row r="102" spans="1:12">
+        <v>0.96924603174603174</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>16</v>
       </c>
@@ -4541,19 +4626,19 @@
         <v>224</v>
       </c>
       <c r="I102">
-        <v>0.7663858794491922</v>
+        <v>0.76638587944919223</v>
       </c>
       <c r="J102">
-        <v>0.7637687433339607</v>
+        <v>0.76376874333396072</v>
       </c>
       <c r="K102">
-        <v>0.8675455116133083</v>
+        <v>0.86754551161330828</v>
       </c>
       <c r="L102">
         <v>0.8747294372294373</v>
       </c>
     </row>
-    <row r="103" spans="1:12">
+    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>16</v>
       </c>
@@ -4579,19 +4664,19 @@
         <v>310</v>
       </c>
       <c r="I103">
-        <v>0.794281454660309</v>
+        <v>0.79428145466030897</v>
       </c>
       <c r="J103">
-        <v>0.8063617541878412</v>
+        <v>0.80636175418784117</v>
       </c>
       <c r="K103">
-        <v>0.8953866146848602</v>
+        <v>0.89538661468486025</v>
       </c>
       <c r="L103">
-        <v>0.9136904761904763</v>
-      </c>
-    </row>
-    <row r="104" spans="1:12">
+        <v>0.91369047619047628</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>16</v>
       </c>
@@ -4617,19 +4702,19 @@
         <v>122</v>
       </c>
       <c r="I104">
-        <v>0.7315249104941142</v>
+        <v>0.73152491049411417</v>
       </c>
       <c r="J104">
-        <v>0.7403751803751805</v>
+        <v>0.74037518037518046</v>
       </c>
       <c r="K104">
-        <v>0.8979687920365885</v>
+        <v>0.89796879203658853</v>
       </c>
       <c r="L104">
-        <v>0.9089556277056278</v>
-      </c>
-    </row>
-    <row r="105" spans="1:12">
+        <v>0.90895562770562777</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>16</v>
       </c>
@@ -4655,19 +4740,19 @@
         <v>139</v>
       </c>
       <c r="I105">
-        <v>0.7316717396785832</v>
+        <v>0.73167173967858323</v>
       </c>
       <c r="J105">
-        <v>0.7532315912750696</v>
+        <v>0.75323159127506956</v>
       </c>
       <c r="K105">
-        <v>0.8846252479912903</v>
+        <v>0.88462524799129028</v>
       </c>
       <c r="L105">
-        <v>0.8985389610389611</v>
-      </c>
-    </row>
-    <row r="106" spans="1:12">
+        <v>0.89853896103896114</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>16</v>
       </c>
@@ -4693,19 +4778,19 @@
         <v>126</v>
       </c>
       <c r="I106">
-        <v>0.7278294449107209</v>
+        <v>0.72782944491072088</v>
       </c>
       <c r="J106">
         <v>0.7391906644080557</v>
       </c>
       <c r="K106">
-        <v>0.8712899153577119</v>
+        <v>0.87128991535771194</v>
       </c>
       <c r="L106">
-        <v>0.8881222943722945</v>
-      </c>
-    </row>
-    <row r="107" spans="1:12">
+        <v>0.88812229437229451</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>16</v>
       </c>
@@ -4731,19 +4816,19 @@
         <v>124</v>
       </c>
       <c r="I107">
-        <v>0.7290931315899816</v>
+        <v>0.72909313158998157</v>
       </c>
       <c r="J107">
-        <v>0.7410985632724763</v>
+        <v>0.74109856327247625</v>
       </c>
       <c r="K107">
-        <v>0.8846252479912903</v>
+        <v>0.88462524799129028</v>
       </c>
       <c r="L107">
-        <v>0.8985389610389611</v>
-      </c>
-    </row>
-    <row r="108" spans="1:12">
+        <v>0.89853896103896114</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>16</v>
       </c>
@@ -4772,16 +4857,16 @@
         <v>0.8365771071165955</v>
       </c>
       <c r="J108">
-        <v>0.8519274376417234</v>
+        <v>0.85192743764172341</v>
       </c>
       <c r="K108">
-        <v>0.8953866146848602</v>
+        <v>0.89538661468486025</v>
       </c>
       <c r="L108">
-        <v>0.9136904761904763</v>
-      </c>
-    </row>
-    <row r="109" spans="1:12">
+        <v>0.91369047619047628</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>16</v>
       </c>
@@ -4813,13 +4898,13 @@
         <v>0.7839356295878035</v>
       </c>
       <c r="K109">
-        <v>0.8953866146848602</v>
+        <v>0.89538661468486025</v>
       </c>
       <c r="L109">
-        <v>0.9136904761904763</v>
-      </c>
-    </row>
-    <row r="110" spans="1:12">
+        <v>0.91369047619047628</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>16</v>
       </c>
@@ -4845,19 +4930,19 @@
         <v>277</v>
       </c>
       <c r="I110">
-        <v>0.7657312770362766</v>
+        <v>0.76573127703627664</v>
       </c>
       <c r="J110">
-        <v>0.7860657596371882</v>
+        <v>0.78606575963718817</v>
       </c>
       <c r="K110">
-        <v>0.8754696725711217</v>
+        <v>0.87546967257112174</v>
       </c>
       <c r="L110">
-        <v>0.8898809523809524</v>
-      </c>
-    </row>
-    <row r="111" spans="1:12">
+        <v>0.88988095238095244</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>16</v>
       </c>
@@ -4886,16 +4971,16 @@
         <v>0.7709368538988729</v>
       </c>
       <c r="J111">
-        <v>0.7598290598290599</v>
+        <v>0.75982905982905991</v>
       </c>
       <c r="K111">
-        <v>0.8076861808044603</v>
+        <v>0.80768618080446031</v>
       </c>
       <c r="L111">
-        <v>0.8214285714285715</v>
-      </c>
-    </row>
-    <row r="112" spans="1:12">
+        <v>0.82142857142857151</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>16</v>
       </c>
@@ -4924,16 +5009,16 @@
         <v>0.7733721517344706</v>
       </c>
       <c r="J112">
-        <v>0.7683760683760684</v>
+        <v>0.76837606837606842</v>
       </c>
       <c r="K112">
-        <v>0.7760683760683761</v>
+        <v>0.77606837606837609</v>
       </c>
       <c r="L112">
-        <v>0.7984126984126984</v>
-      </c>
-    </row>
-    <row r="113" spans="1:12">
+        <v>0.79841269841269835</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>16</v>
       </c>
@@ -4959,19 +5044,19 @@
         <v>42</v>
       </c>
       <c r="I113">
-        <v>0.7552460615069311</v>
+        <v>0.75524606150693108</v>
       </c>
       <c r="J113">
-        <v>0.752020202020202</v>
+        <v>0.75202020202020203</v>
       </c>
       <c r="K113">
-        <v>0.8076861808044603</v>
+        <v>0.80768618080446031</v>
       </c>
       <c r="L113">
-        <v>0.8214285714285715</v>
-      </c>
-    </row>
-    <row r="114" spans="1:12">
+        <v>0.82142857142857151</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>16</v>
       </c>
@@ -4997,19 +5082,19 @@
         <v>56</v>
       </c>
       <c r="I114">
-        <v>0.702612524980341</v>
+        <v>0.70261252498034099</v>
       </c>
       <c r="J114">
-        <v>0.7067521367521368</v>
+        <v>0.70675213675213677</v>
       </c>
       <c r="K114">
-        <v>0.824280697398977</v>
+        <v>0.82428069739897702</v>
       </c>
       <c r="L114">
-        <v>0.8492063492063492</v>
-      </c>
-    </row>
-    <row r="115" spans="1:12">
+        <v>0.84920634920634919</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>16</v>
       </c>
@@ -5038,16 +5123,16 @@
         <v>0.7733721517344706</v>
       </c>
       <c r="J115">
-        <v>0.7683760683760684</v>
+        <v>0.76837606837606842</v>
       </c>
       <c r="K115">
-        <v>0.7693528693528693</v>
+        <v>0.76935286935286928</v>
       </c>
       <c r="L115">
-        <v>0.7984126984126984</v>
-      </c>
-    </row>
-    <row r="116" spans="1:12">
+        <v>0.79841269841269835</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>16</v>
       </c>
@@ -5076,16 +5161,16 @@
         <v>0.7285443722308711</v>
       </c>
       <c r="J116">
-        <v>0.7388888888888889</v>
+        <v>0.73888888888888893</v>
       </c>
       <c r="K116">
-        <v>0.8076861808044603</v>
+        <v>0.80768618080446031</v>
       </c>
       <c r="L116">
-        <v>0.8214285714285715</v>
-      </c>
-    </row>
-    <row r="117" spans="1:12">
+        <v>0.82142857142857151</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>16</v>
       </c>
@@ -5111,19 +5196,19 @@
         <v>91</v>
       </c>
       <c r="I117">
-        <v>0.8168200950954574</v>
+        <v>0.81682009509545739</v>
       </c>
       <c r="J117">
         <v>0.8078282828282829</v>
       </c>
       <c r="K117">
-        <v>0.7844322344322344</v>
+        <v>0.78443223443223442</v>
       </c>
       <c r="L117">
-        <v>0.8531746031746031</v>
-      </c>
-    </row>
-    <row r="118" spans="1:12">
+        <v>0.85317460317460314</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>16</v>
       </c>
@@ -5149,19 +5234,19 @@
         <v>43</v>
       </c>
       <c r="I118">
-        <v>0.7760329906271936</v>
+        <v>0.77603299062719355</v>
       </c>
       <c r="J118">
-        <v>0.7711538461538462</v>
+        <v>0.77115384615384619</v>
       </c>
       <c r="K118">
         <v>0.818131868131868</v>
       </c>
       <c r="L118">
-        <v>0.8206349206349207</v>
-      </c>
-    </row>
-    <row r="119" spans="1:12">
+        <v>0.82063492063492072</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>16</v>
       </c>
@@ -5187,19 +5272,19 @@
         <v>86</v>
       </c>
       <c r="I119">
-        <v>0.7783026538678712</v>
+        <v>0.77830265386787123</v>
       </c>
       <c r="J119">
-        <v>0.7747474747474747</v>
+        <v>0.77474747474747474</v>
       </c>
       <c r="K119">
-        <v>0.830982905982906</v>
+        <v>0.83098290598290603</v>
       </c>
       <c r="L119">
-        <v>0.876984126984127</v>
-      </c>
-    </row>
-    <row r="120" spans="1:12">
+        <v>0.87698412698412698</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>16</v>
       </c>
@@ -5225,19 +5310,19 @@
         <v>87</v>
       </c>
       <c r="I120">
-        <v>0.4378009776118157</v>
+        <v>0.43780097761181569</v>
       </c>
       <c r="J120">
-        <v>0.4391794871794872</v>
+        <v>0.43917948717948718</v>
       </c>
       <c r="K120">
-        <v>0.2594112554112554</v>
+        <v>0.25941125541125543</v>
       </c>
       <c r="L120">
-        <v>0.2692640692640692</v>
-      </c>
-    </row>
-    <row r="121" spans="1:12">
+        <v>0.26926406926406921</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>16</v>
       </c>
@@ -5263,19 +5348,19 @@
         <v>0</v>
       </c>
       <c r="I121">
-        <v>0.3020909846706401</v>
+        <v>0.30209098467064011</v>
       </c>
       <c r="J121">
-        <v>0.3088831908831909</v>
+        <v>0.30888319088319088</v>
       </c>
       <c r="K121">
-        <v>0.172972972972973</v>
+        <v>0.17297297297297301</v>
       </c>
       <c r="L121">
-        <v>0.1939393939393939</v>
-      </c>
-    </row>
-    <row r="122" spans="1:12">
+        <v>0.19393939393939391</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>16</v>
       </c>
@@ -5301,19 +5386,19 @@
         <v>0</v>
       </c>
       <c r="I122">
-        <v>0.2854623225329542</v>
+        <v>0.28546232253295423</v>
       </c>
       <c r="J122">
-        <v>0.2948461538461539</v>
+        <v>0.29484615384615392</v>
       </c>
       <c r="K122">
-        <v>0.1948630136986302</v>
+        <v>0.19486301369863021</v>
       </c>
       <c r="L122">
-        <v>0.2164502164502164</v>
-      </c>
-    </row>
-    <row r="123" spans="1:12">
+        <v>0.21645021645021639</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>16</v>
       </c>
@@ -5339,19 +5424,19 @@
         <v>0</v>
       </c>
       <c r="I123">
-        <v>0.3020909846706401</v>
+        <v>0.30209098467064011</v>
       </c>
       <c r="J123">
-        <v>0.3088831908831909</v>
+        <v>0.30888319088319088</v>
       </c>
       <c r="K123">
-        <v>0.172972972972973</v>
+        <v>0.17297297297297301</v>
       </c>
       <c r="L123">
-        <v>0.1939393939393939</v>
-      </c>
-    </row>
-    <row r="124" spans="1:12">
+        <v>0.19393939393939391</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>16</v>
       </c>
@@ -5377,19 +5462,19 @@
         <v>0</v>
       </c>
       <c r="I124">
-        <v>0.3020909846706401</v>
+        <v>0.30209098467064011</v>
       </c>
       <c r="J124">
-        <v>0.3088831908831909</v>
+        <v>0.30888319088319088</v>
       </c>
       <c r="K124">
-        <v>0.172972972972973</v>
+        <v>0.17297297297297301</v>
       </c>
       <c r="L124">
-        <v>0.1939393939393939</v>
-      </c>
-    </row>
-    <row r="125" spans="1:12">
+        <v>0.19393939393939391</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>16</v>
       </c>
@@ -5418,16 +5503,16 @@
         <v>0.271574399884911</v>
       </c>
       <c r="J125">
-        <v>0.2826905982905983</v>
+        <v>0.28269059829059828</v>
       </c>
       <c r="K125">
-        <v>0.1961389961389962</v>
+        <v>0.19613899613899621</v>
       </c>
       <c r="L125">
-        <v>0.2164502164502164</v>
-      </c>
-    </row>
-    <row r="126" spans="1:12">
+        <v>0.21645021645021639</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>16</v>
       </c>
@@ -5453,19 +5538,19 @@
         <v>83</v>
       </c>
       <c r="I126">
-        <v>0.439297831618248</v>
+        <v>0.43929783161824798</v>
       </c>
       <c r="J126">
-        <v>0.4372</v>
+        <v>0.43719999999999998</v>
       </c>
       <c r="K126">
-        <v>0.2803392041748207</v>
+        <v>0.28033920417482072</v>
       </c>
       <c r="L126">
-        <v>0.2917748917748917</v>
-      </c>
-    </row>
-    <row r="127" spans="1:12">
+        <v>0.29177489177489169</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>16</v>
       </c>
@@ -5491,19 +5576,19 @@
         <v>0</v>
       </c>
       <c r="I127">
-        <v>0.3020909846706401</v>
+        <v>0.30209098467064011</v>
       </c>
       <c r="J127">
-        <v>0.3088831908831909</v>
+        <v>0.30888319088319088</v>
       </c>
       <c r="K127">
-        <v>0.172972972972973</v>
+        <v>0.17297297297297301</v>
       </c>
       <c r="L127">
-        <v>0.1939393939393939</v>
-      </c>
-    </row>
-    <row r="128" spans="1:12">
+        <v>0.19393939393939391</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>16</v>
       </c>
@@ -5532,16 +5617,16 @@
         <v>0.3421138861138861</v>
       </c>
       <c r="J128">
-        <v>0.3489275362318841</v>
+        <v>0.34892753623188411</v>
       </c>
       <c r="K128">
-        <v>0.1984344422700587</v>
+        <v>0.19843444227005869</v>
       </c>
       <c r="L128">
-        <v>0.2164502164502164</v>
-      </c>
-    </row>
-    <row r="129" spans="1:12">
+        <v>0.21645021645021639</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>16</v>
       </c>
@@ -5567,19 +5652,19 @@
         <v>172422</v>
       </c>
       <c r="I129">
-        <v>0.9999490769824009</v>
+        <v>0.99994907698240088</v>
       </c>
       <c r="J129">
-        <v>0.99994907644556</v>
+        <v>0.99994907644555997</v>
       </c>
       <c r="K129">
-        <v>0.8569934609565338</v>
+        <v>0.85699346095653384</v>
       </c>
       <c r="L129">
         <v>0.8571428571428571</v>
       </c>
     </row>
-    <row r="130" spans="1:12">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>16</v>
       </c>
@@ -5605,19 +5690,19 @@
         <v>172422</v>
       </c>
       <c r="I130">
-        <v>0.9999725796658094</v>
+        <v>0.99997257966580944</v>
       </c>
       <c r="J130">
-        <v>0.9999725795584323</v>
+        <v>0.99997257955843233</v>
       </c>
       <c r="K130">
-        <v>0.8548829504460598</v>
+        <v>0.85488295044605978</v>
       </c>
       <c r="L130">
-        <v>0.8570626453838133</v>
-      </c>
-    </row>
-    <row r="131" spans="1:12">
+        <v>0.85706264538381327</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>16</v>
       </c>
@@ -5643,19 +5728,19 @@
         <v>167247</v>
       </c>
       <c r="I131">
-        <v>0.9999959615213725</v>
+        <v>0.99999596152137249</v>
       </c>
       <c r="J131">
         <v>0.9999959615213756</v>
       </c>
       <c r="K131">
-        <v>0.9295955783850388</v>
+        <v>0.92959557838503881</v>
       </c>
       <c r="L131">
-        <v>0.9282567769878686</v>
-      </c>
-    </row>
-    <row r="132" spans="1:12">
+        <v>0.92825677698786857</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>16</v>
       </c>
@@ -5681,19 +5766,19 @@
         <v>135963</v>
       </c>
       <c r="I132">
-        <v>0.9821115199096236</v>
+        <v>0.98211151990962364</v>
       </c>
       <c r="J132">
-        <v>0.9714011512018285</v>
+        <v>0.97140115120182846</v>
       </c>
       <c r="K132">
-        <v>0.8569934609565338</v>
+        <v>0.85699346095653384</v>
       </c>
       <c r="L132">
         <v>0.8571428571428571</v>
       </c>
     </row>
-    <row r="133" spans="1:12">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>16</v>
       </c>
@@ -5719,27 +5804,27 @@
         <v>172422</v>
       </c>
       <c r="I133">
-        <v>0.9999686623371082</v>
+        <v>0.99996866233710824</v>
       </c>
       <c r="J133">
-        <v>0.999968662229737</v>
+        <v>0.99996866222973702</v>
       </c>
       <c r="K133">
-        <v>0.8548829504460598</v>
+        <v>0.85488295044605978</v>
       </c>
       <c r="L133">
-        <v>0.8570626453838133</v>
-      </c>
-    </row>
-    <row r="134" spans="1:12">
+        <v>0.85706264538381327</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B134" t="s">
         <v>20</v>
       </c>
       <c r="C134" t="s">
-        <v>155</v>
+        <v>40</v>
       </c>
       <c r="D134">
         <v>57532</v>
@@ -5750,26 +5835,26 @@
       <c r="F134">
         <v>45932</v>
       </c>
-      <c r="G134">
-        <v>2728</v>
-      </c>
-      <c r="H134">
-        <v>170700</v>
+      <c r="G134" t="s">
+        <v>170</v>
+      </c>
+      <c r="H134" t="s">
+        <v>170</v>
       </c>
       <c r="I134">
-        <v>0.9659527622731439</v>
+        <v>0.93392541375017224</v>
       </c>
       <c r="J134">
-        <v>0.9464008736665506</v>
+        <v>0.90263758856080623</v>
       </c>
       <c r="K134">
-        <v>0.8569934609565338</v>
+        <v>0.83072709611456119</v>
       </c>
       <c r="L134">
-        <v>0.8571428571428571</v>
-      </c>
-    </row>
-    <row r="135" spans="1:12">
+        <v>0.8564822153461753</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>16</v>
       </c>
@@ -5795,19 +5880,19 @@
         <v>163800</v>
       </c>
       <c r="I135">
-        <v>0.9999711366385491</v>
+        <v>0.99997113663854909</v>
       </c>
       <c r="J135">
-        <v>0.9999711366391503</v>
+        <v>0.99997113663915027</v>
       </c>
       <c r="K135">
-        <v>0.9297451419487509</v>
+        <v>0.92974514194875091</v>
       </c>
       <c r="L135">
-        <v>0.9284755474976037</v>
-      </c>
-    </row>
-    <row r="136" spans="1:12">
+        <v>0.92847554749760375</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>16</v>
       </c>
@@ -5833,19 +5918,19 @@
         <v>172422</v>
       </c>
       <c r="I136">
-        <v>0.999960828324136</v>
+        <v>0.99996082832413602</v>
       </c>
       <c r="J136">
-        <v>0.9999608282168209</v>
+        <v>0.99996082821682086</v>
       </c>
       <c r="K136">
-        <v>0.8569934609565338</v>
+        <v>0.85699346095653384</v>
       </c>
       <c r="L136">
         <v>0.8571428571428571</v>
       </c>
     </row>
-    <row r="137" spans="1:12">
+    <row r="137" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>16</v>
       </c>
@@ -5871,19 +5956,19 @@
         <v>155181</v>
       </c>
       <c r="I137">
-        <v>0.9999651801478133</v>
+        <v>0.99996518014781333</v>
       </c>
       <c r="J137">
         <v>0.9999651801492031</v>
       </c>
       <c r="K137">
-        <v>0.9275767926088412</v>
+        <v>0.92757679260884118</v>
       </c>
       <c r="L137">
         <v>0.928379666423779</v>
       </c>
     </row>
-    <row r="138" spans="1:12">
+    <row r="138" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>16</v>
       </c>
@@ -5909,19 +5994,19 @@
         <v>0</v>
       </c>
       <c r="I138">
-        <v>0.7133363542616962</v>
+        <v>0.71333635426169617</v>
       </c>
       <c r="J138">
-        <v>0.6619209039548022</v>
+        <v>0.66192090395480219</v>
       </c>
       <c r="K138">
         <v>0.7652941176470589</v>
       </c>
       <c r="L138">
-        <v>0.7252032520325203</v>
-      </c>
-    </row>
-    <row r="139" spans="1:12">
+        <v>0.72520325203252034</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>16</v>
       </c>
@@ -5947,19 +6032,19 @@
         <v>0</v>
       </c>
       <c r="I139">
-        <v>0.7133363542616962</v>
+        <v>0.71333635426169617</v>
       </c>
       <c r="J139">
-        <v>0.6619209039548022</v>
+        <v>0.66192090395480219</v>
       </c>
       <c r="K139">
         <v>0.7652941176470589</v>
       </c>
       <c r="L139">
-        <v>0.7252032520325203</v>
-      </c>
-    </row>
-    <row r="140" spans="1:12">
+        <v>0.72520325203252034</v>
+      </c>
+    </row>
+    <row r="140" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>16</v>
       </c>
@@ -5985,19 +6070,19 @@
         <v>0</v>
       </c>
       <c r="I140">
-        <v>0.7492074703191335</v>
+        <v>0.74920747031913348</v>
       </c>
       <c r="J140">
-        <v>0.694354920441877</v>
+        <v>0.69435492044187697</v>
       </c>
       <c r="K140">
-        <v>0.7449392712550608</v>
+        <v>0.74493927125506076</v>
       </c>
       <c r="L140">
-        <v>0.733739837398374</v>
-      </c>
-    </row>
-    <row r="141" spans="1:12">
+        <v>0.73373983739837401</v>
+      </c>
+    </row>
+    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>16</v>
       </c>
@@ -6023,19 +6108,19 @@
         <v>0</v>
       </c>
       <c r="I141">
-        <v>0.7133363542616962</v>
+        <v>0.71333635426169617</v>
       </c>
       <c r="J141">
-        <v>0.6619209039548022</v>
+        <v>0.66192090395480219</v>
       </c>
       <c r="K141">
         <v>0.7652941176470589</v>
       </c>
       <c r="L141">
-        <v>0.7252032520325203</v>
-      </c>
-    </row>
-    <row r="142" spans="1:12">
+        <v>0.72520325203252034</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>16</v>
       </c>
@@ -6061,19 +6146,19 @@
         <v>0</v>
       </c>
       <c r="I142">
-        <v>0.7133363542616962</v>
+        <v>0.71333635426169617</v>
       </c>
       <c r="J142">
-        <v>0.6619209039548022</v>
+        <v>0.66192090395480219</v>
       </c>
       <c r="K142">
         <v>0.7652941176470589</v>
       </c>
       <c r="L142">
-        <v>0.7252032520325203</v>
-      </c>
-    </row>
-    <row r="143" spans="1:12">
+        <v>0.72520325203252034</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>16</v>
       </c>
@@ -6099,19 +6184,19 @@
         <v>0</v>
       </c>
       <c r="I143">
-        <v>0.7459922539495089</v>
+        <v>0.74599225394950885</v>
       </c>
       <c r="J143">
         <v>0.6939572165971809</v>
       </c>
       <c r="K143">
-        <v>0.7069520070913005</v>
+        <v>0.70695200709130046</v>
       </c>
       <c r="L143">
-        <v>0.6850948509485095</v>
-      </c>
-    </row>
-    <row r="144" spans="1:12">
+        <v>0.68509485094850953</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>16</v>
       </c>
@@ -6137,19 +6222,19 @@
         <v>1287</v>
       </c>
       <c r="I144">
-        <v>0.9707216859066665</v>
+        <v>0.97072168590666652</v>
       </c>
       <c r="J144">
-        <v>0.9707447890188105</v>
+        <v>0.97074478901881045</v>
       </c>
       <c r="K144">
         <v>0.7503369272237197</v>
       </c>
       <c r="L144">
-        <v>0.7350948509485095</v>
-      </c>
-    </row>
-    <row r="145" spans="1:12">
+        <v>0.73509485094850946</v>
+      </c>
+    </row>
+    <row r="145" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>16</v>
       </c>
@@ -6175,19 +6260,19 @@
         <v>0</v>
       </c>
       <c r="I145">
-        <v>0.7133363542616962</v>
+        <v>0.71333635426169617</v>
       </c>
       <c r="J145">
-        <v>0.6619209039548022</v>
+        <v>0.66192090395480219</v>
       </c>
       <c r="K145">
         <v>0.7652941176470589</v>
       </c>
       <c r="L145">
-        <v>0.7252032520325203</v>
-      </c>
-    </row>
-    <row r="146" spans="1:12">
+        <v>0.72520325203252034</v>
+      </c>
+    </row>
+    <row r="146" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>16</v>
       </c>
@@ -6213,19 +6298,19 @@
         <v>0</v>
       </c>
       <c r="I146">
-        <v>0.7776691926403734</v>
+        <v>0.77766919264037337</v>
       </c>
       <c r="J146">
-        <v>0.7231317143630946</v>
+        <v>0.72313171436309465</v>
       </c>
       <c r="K146">
-        <v>0.7328798185941043</v>
+        <v>0.73287981859410434</v>
       </c>
       <c r="L146">
-        <v>0.7436314363143631</v>
-      </c>
-    </row>
-    <row r="147" spans="1:12">
+        <v>0.74363143631436313</v>
+      </c>
+    </row>
+    <row r="147" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>16</v>
       </c>
@@ -6251,19 +6336,19 @@
         <v>115</v>
       </c>
       <c r="I147">
-        <v>0.9701590932987623</v>
+        <v>0.97015909329876227</v>
       </c>
       <c r="J147">
-        <v>0.9701754385964911</v>
+        <v>0.97017543859649114</v>
       </c>
       <c r="K147">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L147">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="148" spans="1:12">
+    <row r="148" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>16</v>
       </c>
@@ -6289,19 +6374,19 @@
         <v>115</v>
       </c>
       <c r="I148">
-        <v>0.9666511328943079</v>
+        <v>0.96665113289430793</v>
       </c>
       <c r="J148">
-        <v>0.9666666666666666</v>
+        <v>0.96666666666666656</v>
       </c>
       <c r="K148">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L148">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="149" spans="1:12">
+    <row r="149" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>16</v>
       </c>
@@ -6327,19 +6412,19 @@
         <v>112</v>
       </c>
       <c r="I149">
-        <v>0.9728640812561256</v>
+        <v>0.97286408125612556</v>
       </c>
       <c r="J149">
-        <v>0.9728246753246754</v>
+        <v>0.97282467532467543</v>
       </c>
       <c r="K149">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L149">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="150" spans="1:12">
+    <row r="150" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>16</v>
       </c>
@@ -6368,16 +6453,16 @@
         <v>0.9684045735769875</v>
       </c>
       <c r="J150">
-        <v>0.968421052631579</v>
+        <v>0.96842105263157896</v>
       </c>
       <c r="K150">
-        <v>0.9614864864864865</v>
+        <v>0.96148648648648649</v>
       </c>
       <c r="L150">
-        <v>0.9523809523809523</v>
-      </c>
-    </row>
-    <row r="151" spans="1:12">
+        <v>0.95238095238095233</v>
+      </c>
+    </row>
+    <row r="151" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>16</v>
       </c>
@@ -6406,16 +6491,16 @@
         <v>0.9684045735769875</v>
       </c>
       <c r="J151">
-        <v>0.968421052631579</v>
+        <v>0.96842105263157896</v>
       </c>
       <c r="K151">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L151">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="152" spans="1:12">
+    <row r="152" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>16</v>
       </c>
@@ -6441,19 +6526,19 @@
         <v>114</v>
       </c>
       <c r="I152">
-        <v>0.969886682846105</v>
+        <v>0.96988668284610502</v>
       </c>
       <c r="J152">
         <v>0.9698934837092732</v>
       </c>
       <c r="K152">
-        <v>0.9619111259605747</v>
+        <v>0.96191112596057471</v>
       </c>
       <c r="L152">
-        <v>0.9573412698412699</v>
-      </c>
-    </row>
-    <row r="153" spans="1:12">
+        <v>0.95734126984126988</v>
+      </c>
+    </row>
+    <row r="153" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>16</v>
       </c>
@@ -6479,19 +6564,19 @@
         <v>109</v>
       </c>
       <c r="I153">
-        <v>0.9703624264629152</v>
+        <v>0.97036242646291515</v>
       </c>
       <c r="J153">
-        <v>0.9703703703703702</v>
+        <v>0.97037037037037022</v>
       </c>
       <c r="K153">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L153">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="154" spans="1:12">
+    <row r="154" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>16</v>
       </c>
@@ -6517,19 +6602,19 @@
         <v>115</v>
       </c>
       <c r="I154">
-        <v>0.9666535644756868</v>
+        <v>0.96665356447568684</v>
       </c>
       <c r="J154">
-        <v>0.9666666666666666</v>
+        <v>0.96666666666666656</v>
       </c>
       <c r="K154">
-        <v>0.9712773998488284</v>
+        <v>0.97127739984882844</v>
       </c>
       <c r="L154">
         <v>0.9642857142857143</v>
       </c>
     </row>
-    <row r="155" spans="1:12">
+    <row r="155" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>16</v>
       </c>
@@ -6555,16 +6640,319 @@
         <v>103</v>
       </c>
       <c r="I155">
-        <v>0.9784836137695269</v>
+        <v>0.97848361376952686</v>
       </c>
       <c r="J155">
-        <v>0.9784690799396681</v>
+        <v>0.97846907993966814</v>
       </c>
       <c r="K155">
-        <v>0.9619111259605747</v>
+        <v>0.96191112596057471</v>
       </c>
       <c r="L155">
-        <v>0.9573412698412699</v>
+        <v>0.95734126984126988</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L155" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="shuttle"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="adasyn_shuttle_I0_sg208961_train"/>
+        <filter val="borderlinesmote_shuttle_I0_sg172454_train"/>
+        <filter val="PRD20_PR40_CPprop_UD040_Ppp050_I0_SV2096_SG172422"/>
+        <filter val="PRD25_PR70_CPprop_UD055_Ppp055_I0_SV1837_SG172422"/>
+        <filter val="PRD35_PR35_CPent_UD080_PE45_I0_SV1708_SG135963"/>
+        <filter val="PRD35_PR60_CPent_UD050_PE20_I0_SV2939_SG172422"/>
+        <filter val="PRD50_PR30_CPent_UD060_PE30_I0_SV3919_SG172422"/>
+        <filter val="shuttle_I0_tm46400_train"/>
+        <filter val="smote_shuttle_I0_sg208883_train"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A19:L134">
+      <sortCondition descending="1" ref="L1:L155"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9682E1A-ACCB-478C-A091-E84F67832DA5}">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2">
+        <v>35</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F2" s="2">
+        <v>45</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2">
+        <v>40</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>50</v>
+      </c>
+      <c r="C4" s="2">
+        <v>30</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F4" s="2">
+        <v>30</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>35</v>
+      </c>
+      <c r="C5" s="2">
+        <v>60</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F5" s="2">
+        <v>20</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2">
+        <v>70</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>40</v>
+      </c>
+      <c r="C7" s="2">
+        <v>40</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F7" s="2">
+        <v>35</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H7" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>30</v>
+      </c>
+      <c r="C8" s="2">
+        <v>50</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F8" s="2">
+        <v>35</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H8" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>45</v>
+      </c>
+      <c r="C9" s="2">
+        <v>45</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="H9" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>55</v>
+      </c>
+      <c r="C10" s="2">
+        <v>55</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F10" s="2">
+        <v>40</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H10" s="2">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>